<commit_message>
Adding match times to schedule
</commit_message>
<xml_diff>
--- a/WC2026 Data.xlsx
+++ b/WC2026 Data.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16596" windowHeight="5556" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16596" windowHeight="5556"/>
   </bookViews>
   <sheets>
     <sheet name="Teams" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="149">
   <si>
     <t>Groups</t>
   </si>
@@ -132,9 +132,6 @@
     <t>Paraguay</t>
   </si>
   <si>
-    <t>United States of America</t>
-  </si>
-  <si>
     <t>MEX</t>
   </si>
   <si>
@@ -228,9 +225,6 @@
     <t>Portugal</t>
   </si>
   <si>
-    <t>Democratic Republic of the Congo</t>
-  </si>
-  <si>
     <t>Uzbekistan</t>
   </si>
   <si>
@@ -354,9 +348,6 @@
     <t>MAR</t>
   </si>
   <si>
-    <t>CPT</t>
-  </si>
-  <si>
     <t>NZL</t>
   </si>
   <si>
@@ -471,10 +462,16 @@
     <t>Kansas City Stadium</t>
   </si>
   <si>
-    <t>TBD</t>
-  </si>
-  <si>
     <t>Boston Stadium</t>
+  </si>
+  <si>
+    <t>United States</t>
+  </si>
+  <si>
+    <t>DR Congo</t>
+  </si>
+  <si>
+    <t>CPV</t>
   </si>
 </sst>
 </file>
@@ -510,9 +507,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -838,25 +836,25 @@
         <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D2" t="s">
         <v>22</v>
       </c>
       <c r="E2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
         <v>23</v>
       </c>
       <c r="G2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H2" t="s">
         <v>24</v>
       </c>
       <c r="I2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -867,25 +865,25 @@
         <v>25</v>
       </c>
       <c r="C3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D3" t="s">
         <v>26</v>
       </c>
       <c r="E3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="F3" t="s">
         <v>27</v>
       </c>
       <c r="G3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H3" t="s">
         <v>28</v>
       </c>
       <c r="I3" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -896,25 +894,25 @@
         <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
         <v>30</v>
       </c>
       <c r="E4" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F4" t="s">
         <v>31</v>
       </c>
       <c r="G4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="H4" t="s">
         <v>32</v>
       </c>
       <c r="I4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -922,7 +920,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>146</v>
       </c>
       <c r="C5" t="s">
         <v>33</v>
@@ -931,19 +929,19 @@
         <v>34</v>
       </c>
       <c r="E5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" t="s">
         <v>40</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
+        <v>86</v>
+      </c>
+      <c r="H5" t="s">
         <v>41</v>
       </c>
-      <c r="G5" t="s">
-        <v>88</v>
-      </c>
-      <c r="H5" t="s">
-        <v>42</v>
-      </c>
       <c r="I5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -951,28 +949,28 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" t="s">
+        <v>90</v>
+      </c>
+      <c r="D6" t="s">
         <v>43</v>
       </c>
-      <c r="C6" t="s">
-        <v>92</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
+        <v>109</v>
+      </c>
+      <c r="F6" t="s">
+        <v>133</v>
+      </c>
+      <c r="G6" t="s">
+        <v>101</v>
+      </c>
+      <c r="H6" t="s">
         <v>44</v>
       </c>
-      <c r="E6" t="s">
-        <v>112</v>
-      </c>
-      <c r="F6" t="s">
-        <v>136</v>
-      </c>
-      <c r="G6" t="s">
-        <v>103</v>
-      </c>
-      <c r="H6" t="s">
-        <v>45</v>
-      </c>
       <c r="I6" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -980,28 +978,28 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" t="s">
+        <v>95</v>
+      </c>
+      <c r="D7" t="s">
         <v>46</v>
       </c>
-      <c r="C7" t="s">
-        <v>97</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
+        <v>98</v>
+      </c>
+      <c r="F7" t="s">
         <v>47</v>
       </c>
-      <c r="E7" t="s">
-        <v>100</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
+        <v>87</v>
+      </c>
+      <c r="H7" t="s">
         <v>48</v>
       </c>
-      <c r="G7" t="s">
-        <v>89</v>
-      </c>
-      <c r="H7" t="s">
-        <v>49</v>
-      </c>
       <c r="I7" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
@@ -1009,28 +1007,28 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" t="s">
+        <v>91</v>
+      </c>
+      <c r="D8" t="s">
         <v>50</v>
       </c>
-      <c r="C8" t="s">
-        <v>93</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
+        <v>103</v>
+      </c>
+      <c r="F8" t="s">
         <v>51</v>
       </c>
-      <c r="E8" t="s">
-        <v>105</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
+        <v>96</v>
+      </c>
+      <c r="H8" t="s">
         <v>52</v>
       </c>
-      <c r="G8" t="s">
-        <v>98</v>
-      </c>
-      <c r="H8" t="s">
-        <v>53</v>
-      </c>
       <c r="I8" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -1038,28 +1036,28 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" t="s">
+        <v>111</v>
+      </c>
+      <c r="D9" t="s">
         <v>54</v>
       </c>
-      <c r="C9" t="s">
-        <v>114</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
+        <v>148</v>
+      </c>
+      <c r="F9" t="s">
         <v>55</v>
       </c>
-      <c r="E9" t="s">
-        <v>109</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
+        <v>99</v>
+      </c>
+      <c r="H9" t="s">
         <v>56</v>
       </c>
-      <c r="G9" t="s">
-        <v>101</v>
-      </c>
-      <c r="H9" t="s">
-        <v>57</v>
-      </c>
       <c r="I9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -1067,28 +1065,28 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10" t="s">
+        <v>92</v>
+      </c>
+      <c r="D10" t="s">
         <v>58</v>
       </c>
-      <c r="C10" t="s">
-        <v>94</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F10" t="s">
         <v>59</v>
       </c>
-      <c r="E10" t="s">
-        <v>106</v>
-      </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
+        <v>97</v>
+      </c>
+      <c r="H10" t="s">
         <v>60</v>
       </c>
-      <c r="G10" t="s">
-        <v>99</v>
-      </c>
-      <c r="H10" t="s">
-        <v>61</v>
-      </c>
       <c r="I10" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
@@ -1096,28 +1094,28 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" t="s">
+        <v>89</v>
+      </c>
+      <c r="D11" t="s">
         <v>62</v>
       </c>
-      <c r="C11" t="s">
-        <v>91</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
+        <v>100</v>
+      </c>
+      <c r="F11" t="s">
         <v>63</v>
       </c>
-      <c r="E11" t="s">
-        <v>102</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
+        <v>112</v>
+      </c>
+      <c r="H11" t="s">
         <v>64</v>
       </c>
-      <c r="G11" t="s">
-        <v>115</v>
-      </c>
-      <c r="H11" t="s">
-        <v>65</v>
-      </c>
       <c r="I11" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
@@ -1125,28 +1123,28 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D12" t="s">
+        <v>147</v>
+      </c>
+      <c r="E12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F12" t="s">
         <v>66</v>
       </c>
-      <c r="C12" t="s">
-        <v>95</v>
-      </c>
-      <c r="D12" t="s">
+      <c r="G12" t="s">
+        <v>88</v>
+      </c>
+      <c r="H12" t="s">
         <v>67</v>
       </c>
-      <c r="E12" t="s">
-        <v>104</v>
-      </c>
-      <c r="F12" t="s">
-        <v>68</v>
-      </c>
-      <c r="G12" t="s">
-        <v>90</v>
-      </c>
-      <c r="H12" t="s">
-        <v>69</v>
-      </c>
       <c r="I12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
@@ -1154,28 +1152,28 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" t="s">
+        <v>94</v>
+      </c>
+      <c r="D13" t="s">
+        <v>69</v>
+      </c>
+      <c r="E13" t="s">
+        <v>105</v>
+      </c>
+      <c r="F13" t="s">
         <v>70</v>
       </c>
-      <c r="C13" t="s">
-        <v>96</v>
-      </c>
-      <c r="D13" t="s">
+      <c r="G13" t="s">
+        <v>75</v>
+      </c>
+      <c r="H13" t="s">
         <v>71</v>
       </c>
-      <c r="E13" t="s">
-        <v>107</v>
-      </c>
-      <c r="F13" t="s">
-        <v>72</v>
-      </c>
-      <c r="G13" t="s">
-        <v>77</v>
-      </c>
-      <c r="H13" t="s">
-        <v>73</v>
-      </c>
       <c r="I13" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -1194,7 +1192,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B1" t="s">
         <v>13</v>
@@ -1203,13 +1201,13 @@
         <v>14</v>
       </c>
       <c r="D1" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="E1" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="F1" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -1217,19 +1215,19 @@
         <v>46184</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E2" t="s">
-        <v>120</v>
-      </c>
-      <c r="F2" t="s">
-        <v>148</v>
+        <v>117</v>
+      </c>
+      <c r="F2" s="2">
+        <v>0.58333333333333337</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -1237,19 +1235,19 @@
         <v>46184</v>
       </c>
       <c r="B3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D3" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E3" t="s">
-        <v>121</v>
-      </c>
-      <c r="F3" t="s">
-        <v>148</v>
+        <v>118</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0.875</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -1257,19 +1255,19 @@
         <v>46185</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="D4" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E4" t="s">
-        <v>123</v>
-      </c>
-      <c r="F4" t="s">
-        <v>148</v>
+        <v>120</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0.58333333333333337</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -1280,16 +1278,16 @@
         <v>33</v>
       </c>
       <c r="C5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E5" t="s">
-        <v>125</v>
-      </c>
-      <c r="F5" t="s">
-        <v>148</v>
+        <v>122</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0.83333333333333337</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -1297,19 +1295,19 @@
         <v>46186</v>
       </c>
       <c r="B6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C6" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D6" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="E6" t="s">
-        <v>149</v>
-      </c>
-      <c r="F6" t="s">
-        <v>148</v>
+        <v>145</v>
+      </c>
+      <c r="F6" s="2">
+        <v>0.83333333333333337</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -1317,19 +1315,19 @@
         <v>46186</v>
       </c>
       <c r="B7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C7" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E7" t="s">
-        <v>137</v>
-      </c>
-      <c r="F7" t="s">
-        <v>148</v>
+        <v>134</v>
+      </c>
+      <c r="F7" s="2">
+        <v>0.95833333333333337</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -1337,19 +1335,19 @@
         <v>46186</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D8" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="E8" t="s">
-        <v>138</v>
-      </c>
-      <c r="F8" t="s">
-        <v>148</v>
+        <v>135</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -1357,19 +1355,19 @@
         <v>46186</v>
       </c>
       <c r="B9" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C9" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="D9" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E9" t="s">
-        <v>139</v>
-      </c>
-      <c r="F9" t="s">
-        <v>148</v>
+        <v>136</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0.58333333333333337</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -1377,19 +1375,19 @@
         <v>46187</v>
       </c>
       <c r="B10" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C10" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D10" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E10" t="s">
-        <v>140</v>
-      </c>
-      <c r="F10" t="s">
-        <v>148</v>
+        <v>137</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0.75</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -1397,19 +1395,19 @@
         <v>46187</v>
       </c>
       <c r="B11" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C11" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D11" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E11" t="s">
-        <v>141</v>
-      </c>
-      <c r="F11" t="s">
-        <v>148</v>
+        <v>138</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0.5</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -1417,19 +1415,19 @@
         <v>46187</v>
       </c>
       <c r="B12" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C12" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D12" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E12" t="s">
-        <v>142</v>
-      </c>
-      <c r="F12" t="s">
-        <v>148</v>
+        <v>139</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0.625</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -1437,19 +1435,19 @@
         <v>46187</v>
       </c>
       <c r="B13" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C13" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D13" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E13" t="s">
-        <v>143</v>
-      </c>
-      <c r="F13" t="s">
-        <v>148</v>
+        <v>140</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0.875</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -1457,19 +1455,19 @@
         <v>46188</v>
       </c>
       <c r="B14" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C14" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D14" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="E14" t="s">
-        <v>144</v>
-      </c>
-      <c r="F14" t="s">
-        <v>148</v>
+        <v>141</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -1477,19 +1475,19 @@
         <v>46188</v>
       </c>
       <c r="B15" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C15" t="s">
-        <v>109</v>
+        <v>148</v>
       </c>
       <c r="D15" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="E15" t="s">
-        <v>145</v>
-      </c>
-      <c r="F15" t="s">
-        <v>148</v>
+        <v>142</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0.45833333333333331</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -1497,19 +1495,19 @@
         <v>46188</v>
       </c>
       <c r="B16" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C16" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D16" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="E16" t="s">
-        <v>125</v>
-      </c>
-      <c r="F16" t="s">
-        <v>148</v>
+        <v>122</v>
+      </c>
+      <c r="F16" s="2">
+        <v>0.83333333333333337</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
@@ -1517,19 +1515,19 @@
         <v>46188</v>
       </c>
       <c r="B17" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C17" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D17" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="E17" t="s">
-        <v>146</v>
-      </c>
-      <c r="F17" t="s">
-        <v>148</v>
+        <v>143</v>
+      </c>
+      <c r="F17" s="2">
+        <v>0.58333333333333337</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
@@ -1537,19 +1535,19 @@
         <v>46189</v>
       </c>
       <c r="B18" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C18" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D18" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E18" t="s">
-        <v>138</v>
-      </c>
-      <c r="F18" t="s">
-        <v>148</v>
+        <v>135</v>
+      </c>
+      <c r="F18" s="2">
+        <v>0.58333333333333337</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -1557,19 +1555,19 @@
         <v>46189</v>
       </c>
       <c r="B19" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C19" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D19" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E19" t="s">
-        <v>149</v>
-      </c>
-      <c r="F19" t="s">
-        <v>148</v>
+        <v>145</v>
+      </c>
+      <c r="F19" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
@@ -1577,19 +1575,19 @@
         <v>46189</v>
       </c>
       <c r="B20" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C20" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D20" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="E20" t="s">
-        <v>147</v>
-      </c>
-      <c r="F20" t="s">
-        <v>148</v>
+        <v>144</v>
+      </c>
+      <c r="F20" s="2">
+        <v>0.83333333333333337</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -1597,19 +1595,19 @@
         <v>46189</v>
       </c>
       <c r="B21" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C21" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D21" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="E21" t="s">
-        <v>139</v>
-      </c>
-      <c r="F21" t="s">
-        <v>148</v>
+        <v>136</v>
+      </c>
+      <c r="F21" s="2">
+        <v>0.95833333333333337</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -1617,19 +1615,19 @@
         <v>46190</v>
       </c>
       <c r="B22" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C22" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D22" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E22" t="s">
-        <v>123</v>
-      </c>
-      <c r="F22" t="s">
-        <v>148</v>
+        <v>120</v>
+      </c>
+      <c r="F22" s="2">
+        <v>0.75</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
@@ -1637,19 +1635,19 @@
         <v>46190</v>
       </c>
       <c r="B23" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C23" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D23" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E23" t="s">
-        <v>142</v>
-      </c>
-      <c r="F23" t="s">
-        <v>148</v>
+        <v>139</v>
+      </c>
+      <c r="F23" s="2">
+        <v>0.625</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -1657,19 +1655,19 @@
         <v>46190</v>
       </c>
       <c r="B24" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C24" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D24" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E24" t="s">
-        <v>141</v>
-      </c>
-      <c r="F24" t="s">
-        <v>148</v>
+        <v>138</v>
+      </c>
+      <c r="F24" s="2">
+        <v>0.5</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
@@ -1677,19 +1675,19 @@
         <v>46190</v>
       </c>
       <c r="B25" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C25" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D25" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E25" t="s">
-        <v>120</v>
-      </c>
-      <c r="F25" t="s">
-        <v>148</v>
+        <v>117</v>
+      </c>
+      <c r="F25" s="2">
+        <v>0.875</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
@@ -1697,19 +1695,19 @@
         <v>46191</v>
       </c>
       <c r="B26" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C26" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D26" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E26" t="s">
-        <v>145</v>
-      </c>
-      <c r="F26" t="s">
-        <v>148</v>
+        <v>142</v>
+      </c>
+      <c r="F26" s="2">
+        <v>0.45833333333333331</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
@@ -1717,19 +1715,19 @@
         <v>46191</v>
       </c>
       <c r="B27" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C27" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="D27" t="s">
+        <v>119</v>
+      </c>
+      <c r="E27" t="s">
         <v>122</v>
       </c>
-      <c r="E27" t="s">
-        <v>125</v>
-      </c>
-      <c r="F27" t="s">
-        <v>148</v>
+      <c r="F27" s="2">
+        <v>0.58333333333333337</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
@@ -1737,19 +1735,19 @@
         <v>46191</v>
       </c>
       <c r="B28" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C28" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D28" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E28" t="s">
-        <v>137</v>
-      </c>
-      <c r="F28" t="s">
-        <v>148</v>
+        <v>134</v>
+      </c>
+      <c r="F28" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
@@ -1757,19 +1755,19 @@
         <v>46191</v>
       </c>
       <c r="B29" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C29" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D29" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E29" t="s">
-        <v>121</v>
-      </c>
-      <c r="F29" t="s">
-        <v>148</v>
+        <v>118</v>
+      </c>
+      <c r="F29" s="2">
+        <v>0.83333333333333337</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
@@ -1777,19 +1775,19 @@
         <v>46192</v>
       </c>
       <c r="B30" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C30" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D30" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="E30" t="s">
-        <v>140</v>
-      </c>
-      <c r="F30" t="s">
-        <v>148</v>
+        <v>137</v>
+      </c>
+      <c r="F30" s="2">
+        <v>0.8125</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
@@ -1797,19 +1795,19 @@
         <v>46192</v>
       </c>
       <c r="B31" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C31" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D31" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="E31" t="s">
-        <v>149</v>
-      </c>
-      <c r="F31" t="s">
-        <v>148</v>
+        <v>145</v>
+      </c>
+      <c r="F31" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
@@ -1817,19 +1815,19 @@
         <v>46192</v>
       </c>
       <c r="B32" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C32" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D32" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E32" t="s">
-        <v>139</v>
-      </c>
-      <c r="F32" t="s">
-        <v>148</v>
+        <v>136</v>
+      </c>
+      <c r="F32" s="2">
+        <v>0.91666666666666663</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
@@ -1840,16 +1838,16 @@
         <v>33</v>
       </c>
       <c r="C33" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D33" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E33" t="s">
-        <v>146</v>
-      </c>
-      <c r="F33" t="s">
-        <v>148</v>
+        <v>143</v>
+      </c>
+      <c r="F33" s="2">
+        <v>0.58333333333333337</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
@@ -1857,19 +1855,19 @@
         <v>46193</v>
       </c>
       <c r="B34" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C34" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D34" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E34" t="s">
-        <v>123</v>
-      </c>
-      <c r="F34" t="s">
-        <v>148</v>
+        <v>120</v>
+      </c>
+      <c r="F34" s="2">
+        <v>0.625</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
@@ -1877,19 +1875,19 @@
         <v>46193</v>
       </c>
       <c r="B35" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C35" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D35" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E35" t="s">
-        <v>147</v>
-      </c>
-      <c r="F35" t="s">
-        <v>148</v>
+        <v>144</v>
+      </c>
+      <c r="F35" s="2">
+        <v>0.79166666666666663</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
@@ -1897,19 +1895,19 @@
         <v>46193</v>
       </c>
       <c r="B36" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C36" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D36" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E36" t="s">
-        <v>141</v>
-      </c>
-      <c r="F36" t="s">
-        <v>148</v>
+        <v>138</v>
+      </c>
+      <c r="F36" s="2">
+        <v>0.5</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
@@ -1917,19 +1915,19 @@
         <v>46193</v>
       </c>
       <c r="B37" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C37" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D37" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E37" t="s">
-        <v>143</v>
-      </c>
-      <c r="F37" t="s">
-        <v>148</v>
+        <v>140</v>
+      </c>
+      <c r="F37" s="2">
+        <v>0.95833333333333337</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
@@ -1937,19 +1935,19 @@
         <v>46194</v>
       </c>
       <c r="B38" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C38" t="s">
-        <v>109</v>
+        <v>148</v>
       </c>
       <c r="D38" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="E38" t="s">
-        <v>144</v>
-      </c>
-      <c r="F38" t="s">
-        <v>148</v>
+        <v>141</v>
+      </c>
+      <c r="F38" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
@@ -1957,19 +1955,19 @@
         <v>46194</v>
       </c>
       <c r="B39" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C39" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D39" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="E39" t="s">
-        <v>145</v>
-      </c>
-      <c r="F39" t="s">
-        <v>148</v>
+        <v>142</v>
+      </c>
+      <c r="F39" s="2">
+        <v>0.45833333333333331</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
@@ -1977,19 +1975,19 @@
         <v>46194</v>
       </c>
       <c r="B40" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C40" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D40" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="E40" t="s">
-        <v>125</v>
-      </c>
-      <c r="F40" t="s">
-        <v>148</v>
+        <v>122</v>
+      </c>
+      <c r="F40" s="2">
+        <v>0.58333333333333337</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
@@ -1997,19 +1995,19 @@
         <v>46194</v>
       </c>
       <c r="B41" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C41" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D41" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="E41" t="s">
-        <v>137</v>
-      </c>
-      <c r="F41" t="s">
-        <v>148</v>
+        <v>134</v>
+      </c>
+      <c r="F41" s="2">
+        <v>0.83333333333333337</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
@@ -2017,19 +2015,19 @@
         <v>46195</v>
       </c>
       <c r="B42" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C42" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D42" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E42" t="s">
-        <v>138</v>
-      </c>
-      <c r="F42" t="s">
-        <v>148</v>
+        <v>135</v>
+      </c>
+      <c r="F42" s="2">
+        <v>0.79166666666666663</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
@@ -2037,19 +2035,19 @@
         <v>46195</v>
       </c>
       <c r="B43" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C43" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D43" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E43" t="s">
-        <v>140</v>
-      </c>
-      <c r="F43" t="s">
-        <v>148</v>
+        <v>137</v>
+      </c>
+      <c r="F43" s="2">
+        <v>0.66666666666666663</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
@@ -2057,19 +2055,19 @@
         <v>46195</v>
       </c>
       <c r="B44" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C44" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D44" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="E44" t="s">
-        <v>142</v>
-      </c>
-      <c r="F44" t="s">
-        <v>148</v>
+        <v>139</v>
+      </c>
+      <c r="F44" s="2">
+        <v>0.5</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
@@ -2077,19 +2075,19 @@
         <v>46195</v>
       </c>
       <c r="B45" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C45" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D45" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="E45" t="s">
-        <v>139</v>
-      </c>
-      <c r="F45" t="s">
-        <v>148</v>
+        <v>136</v>
+      </c>
+      <c r="F45" s="2">
+        <v>0.91666666666666663</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -2097,19 +2095,19 @@
         <v>46196</v>
       </c>
       <c r="B46" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C46" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D46" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E46" t="s">
-        <v>149</v>
-      </c>
-      <c r="F46" t="s">
-        <v>148</v>
+        <v>145</v>
+      </c>
+      <c r="F46" s="2">
+        <v>0.625</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
@@ -2117,19 +2115,19 @@
         <v>46196</v>
       </c>
       <c r="B47" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C47" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D47" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E47" t="s">
-        <v>123</v>
-      </c>
-      <c r="F47" t="s">
-        <v>148</v>
+        <v>120</v>
+      </c>
+      <c r="F47" s="2">
+        <v>0.75</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
@@ -2137,19 +2135,19 @@
         <v>46196</v>
       </c>
       <c r="B48" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C48" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D48" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E48" t="s">
-        <v>141</v>
-      </c>
-      <c r="F48" t="s">
-        <v>148</v>
+        <v>138</v>
+      </c>
+      <c r="F48" s="2">
+        <v>0.5</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -2157,19 +2155,19 @@
         <v>46196</v>
       </c>
       <c r="B49" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C49" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D49" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E49" t="s">
-        <v>121</v>
-      </c>
-      <c r="F49" t="s">
-        <v>148</v>
+        <v>118</v>
+      </c>
+      <c r="F49" s="2">
+        <v>0.875</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
@@ -2177,19 +2175,19 @@
         <v>46197</v>
       </c>
       <c r="B50" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C50" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D50" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="E50" t="s">
-        <v>144</v>
-      </c>
-      <c r="F50" t="s">
-        <v>148</v>
+        <v>141</v>
+      </c>
+      <c r="F50" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
@@ -2197,19 +2195,19 @@
         <v>46197</v>
       </c>
       <c r="B51" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C51" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D51" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="E51" t="s">
-        <v>145</v>
-      </c>
-      <c r="F51" t="s">
-        <v>148</v>
+        <v>142</v>
+      </c>
+      <c r="F51" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
@@ -2217,19 +2215,19 @@
         <v>46197</v>
       </c>
       <c r="B52" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C52" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D52" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E52" t="s">
-        <v>137</v>
-      </c>
-      <c r="F52" t="s">
-        <v>148</v>
+        <v>134</v>
+      </c>
+      <c r="F52" s="2">
+        <v>0.58333333333333337</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
@@ -2237,19 +2235,19 @@
         <v>46197</v>
       </c>
       <c r="B53" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C53" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D53" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E53" t="s">
-        <v>146</v>
-      </c>
-      <c r="F53" t="s">
-        <v>148</v>
+        <v>143</v>
+      </c>
+      <c r="F53" s="2">
+        <v>0.58333333333333337</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
@@ -2257,19 +2255,19 @@
         <v>46197</v>
       </c>
       <c r="B54" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C54" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D54" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E54" t="s">
-        <v>120</v>
-      </c>
-      <c r="F54" t="s">
-        <v>148</v>
+        <v>117</v>
+      </c>
+      <c r="F54" s="2">
+        <v>0.83333333333333337</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
@@ -2277,19 +2275,19 @@
         <v>46197</v>
       </c>
       <c r="B55" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C55" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D55" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E55" t="s">
-        <v>143</v>
-      </c>
-      <c r="F55" t="s">
-        <v>148</v>
+        <v>140</v>
+      </c>
+      <c r="F55" s="2">
+        <v>0.83333333333333337</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
@@ -2297,19 +2295,19 @@
         <v>46198</v>
       </c>
       <c r="B56" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C56" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D56" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E56" t="s">
-        <v>140</v>
-      </c>
-      <c r="F56" t="s">
-        <v>148</v>
+        <v>137</v>
+      </c>
+      <c r="F56" s="2">
+        <v>0.625</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
@@ -2317,19 +2315,19 @@
         <v>46198</v>
       </c>
       <c r="B57" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C57" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D57" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E57" t="s">
-        <v>138</v>
-      </c>
-      <c r="F57" t="s">
-        <v>148</v>
+        <v>135</v>
+      </c>
+      <c r="F57" s="2">
+        <v>0.625</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
@@ -2337,19 +2335,19 @@
         <v>46198</v>
       </c>
       <c r="B58" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C58" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D58" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E58" t="s">
-        <v>142</v>
-      </c>
-      <c r="F58" t="s">
-        <v>148</v>
+        <v>139</v>
+      </c>
+      <c r="F58" s="2">
+        <v>0.75</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
@@ -2357,19 +2355,19 @@
         <v>46198</v>
       </c>
       <c r="B59" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C59" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D59" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E59" t="s">
-        <v>147</v>
-      </c>
-      <c r="F59" t="s">
-        <v>148</v>
+        <v>144</v>
+      </c>
+      <c r="F59" s="2">
+        <v>0.75</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
@@ -2377,19 +2375,19 @@
         <v>46198</v>
       </c>
       <c r="B60" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C60" t="s">
         <v>33</v>
       </c>
       <c r="D60" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E60" t="s">
-        <v>125</v>
-      </c>
-      <c r="F60" t="s">
-        <v>148</v>
+        <v>122</v>
+      </c>
+      <c r="F60" s="2">
+        <v>0.875</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
@@ -2397,19 +2395,19 @@
         <v>46198</v>
       </c>
       <c r="B61" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C61" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D61" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E61" t="s">
-        <v>139</v>
-      </c>
-      <c r="F61" t="s">
-        <v>148</v>
+        <v>136</v>
+      </c>
+      <c r="F61" s="2">
+        <v>0.875</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
@@ -2417,19 +2415,19 @@
         <v>46199</v>
       </c>
       <c r="B62" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C62" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D62" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E62" t="s">
-        <v>149</v>
-      </c>
-      <c r="F62" t="s">
-        <v>148</v>
+        <v>145</v>
+      </c>
+      <c r="F62" s="2">
+        <v>0.58333333333333337</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
@@ -2437,19 +2435,19 @@
         <v>46199</v>
       </c>
       <c r="B63" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C63" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D63" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E63" t="s">
-        <v>123</v>
-      </c>
-      <c r="F63" t="s">
-        <v>148</v>
+        <v>120</v>
+      </c>
+      <c r="F63" s="2">
+        <v>0.58333333333333337</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
@@ -2457,19 +2455,19 @@
         <v>46199</v>
       </c>
       <c r="B64" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C64" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D64" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="E64" t="s">
-        <v>146</v>
-      </c>
-      <c r="F64" t="s">
-        <v>148</v>
+        <v>143</v>
+      </c>
+      <c r="F64" s="2">
+        <v>0.91666666666666663</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
@@ -2477,19 +2475,19 @@
         <v>46199</v>
       </c>
       <c r="B65" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C65" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D65" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="E65" t="s">
-        <v>137</v>
-      </c>
-      <c r="F65" t="s">
-        <v>148</v>
+        <v>134</v>
+      </c>
+      <c r="F65" s="2">
+        <v>0.91666666666666663</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
@@ -2497,19 +2495,19 @@
         <v>46199</v>
       </c>
       <c r="B66" t="s">
-        <v>109</v>
+        <v>148</v>
       </c>
       <c r="C66" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D66" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="E66" t="s">
-        <v>141</v>
-      </c>
-      <c r="F66" t="s">
-        <v>148</v>
+        <v>138</v>
+      </c>
+      <c r="F66" s="2">
+        <v>0.79166666666666663</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
@@ -2517,19 +2515,19 @@
         <v>46199</v>
       </c>
       <c r="B67" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C67" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D67" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="E67" t="s">
-        <v>121</v>
-      </c>
-      <c r="F67" t="s">
-        <v>148</v>
+        <v>118</v>
+      </c>
+      <c r="F67" s="2">
+        <v>0.79166666666666663</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
@@ -2537,19 +2535,19 @@
         <v>46200</v>
       </c>
       <c r="B68" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C68" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D68" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E68" t="s">
-        <v>138</v>
-      </c>
-      <c r="F68" t="s">
-        <v>148</v>
+        <v>135</v>
+      </c>
+      <c r="F68" s="2">
+        <v>0.66666666666666663</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
@@ -2557,19 +2555,19 @@
         <v>46200</v>
       </c>
       <c r="B69" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C69" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D69" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E69" t="s">
-        <v>140</v>
-      </c>
-      <c r="F69" t="s">
-        <v>148</v>
+        <v>137</v>
+      </c>
+      <c r="F69" s="2">
+        <v>0.66666666666666663</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
@@ -2577,19 +2575,19 @@
         <v>46200</v>
       </c>
       <c r="B70" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C70" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D70" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="E70" t="s">
-        <v>147</v>
-      </c>
-      <c r="F70" t="s">
-        <v>148</v>
+        <v>144</v>
+      </c>
+      <c r="F70" s="2">
+        <v>0.875</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
@@ -2597,19 +2595,19 @@
         <v>46200</v>
       </c>
       <c r="B71" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C71" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D71" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="E71" t="s">
-        <v>142</v>
-      </c>
-      <c r="F71" t="s">
-        <v>148</v>
+        <v>139</v>
+      </c>
+      <c r="F71" s="2">
+        <v>0.875</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
@@ -2617,19 +2615,19 @@
         <v>46200</v>
       </c>
       <c r="B72" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C72" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D72" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E72" t="s">
-        <v>144</v>
-      </c>
-      <c r="F72" t="s">
-        <v>148</v>
+        <v>141</v>
+      </c>
+      <c r="F72" s="2">
+        <v>0.77083333333333337</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
@@ -2637,19 +2635,19 @@
         <v>46200</v>
       </c>
       <c r="B73" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C73" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D73" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E73" t="s">
-        <v>145</v>
-      </c>
-      <c r="F73" t="s">
-        <v>148</v>
+        <v>142</v>
+      </c>
+      <c r="F73" s="2">
+        <v>0.77083333333333337</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updating site data and teams page
</commit_message>
<xml_diff>
--- a/WC2026 Data.xlsx
+++ b/WC2026 Data.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16596" windowHeight="5556"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16596" windowHeight="5556" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Teams" sheetId="1" r:id="rId1"/>
@@ -228,9 +228,6 @@
     <t>Uzbekistan</t>
   </si>
   <si>
-    <t>Columbia</t>
-  </si>
-  <si>
     <t>England</t>
   </si>
   <si>
@@ -472,6 +469,9 @@
   </si>
   <si>
     <t>CPV</t>
+  </si>
+  <si>
+    <t>Colombia</t>
   </si>
 </sst>
 </file>
@@ -848,13 +848,13 @@
         <v>23</v>
       </c>
       <c r="G2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H2" t="s">
         <v>24</v>
       </c>
       <c r="I2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -871,19 +871,19 @@
         <v>26</v>
       </c>
       <c r="E3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F3" t="s">
         <v>27</v>
       </c>
       <c r="G3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H3" t="s">
         <v>28</v>
       </c>
       <c r="I3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -900,19 +900,19 @@
         <v>30</v>
       </c>
       <c r="E4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F4" t="s">
         <v>31</v>
       </c>
       <c r="G4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H4" t="s">
         <v>32</v>
       </c>
       <c r="I4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -920,7 +920,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C5" t="s">
         <v>33</v>
@@ -935,13 +935,13 @@
         <v>40</v>
       </c>
       <c r="G5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H5" t="s">
         <v>41</v>
       </c>
       <c r="I5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -952,25 +952,25 @@
         <v>42</v>
       </c>
       <c r="C6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D6" t="s">
         <v>43</v>
       </c>
       <c r="E6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H6" t="s">
         <v>44</v>
       </c>
       <c r="I6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -981,25 +981,25 @@
         <v>45</v>
       </c>
       <c r="C7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D7" t="s">
         <v>46</v>
       </c>
       <c r="E7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F7" t="s">
         <v>47</v>
       </c>
       <c r="G7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H7" t="s">
         <v>48</v>
       </c>
       <c r="I7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
@@ -1010,25 +1010,25 @@
         <v>49</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D8" t="s">
         <v>50</v>
       </c>
       <c r="E8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F8" t="s">
         <v>51</v>
       </c>
       <c r="G8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H8" t="s">
         <v>52</v>
       </c>
       <c r="I8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -1039,25 +1039,25 @@
         <v>53</v>
       </c>
       <c r="C9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D9" t="s">
         <v>54</v>
       </c>
       <c r="E9" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F9" t="s">
         <v>55</v>
       </c>
       <c r="G9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H9" t="s">
         <v>56</v>
       </c>
       <c r="I9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -1068,25 +1068,25 @@
         <v>57</v>
       </c>
       <c r="C10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D10" t="s">
         <v>58</v>
       </c>
       <c r="E10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F10" t="s">
         <v>59</v>
       </c>
       <c r="G10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H10" t="s">
         <v>60</v>
       </c>
       <c r="I10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
@@ -1097,25 +1097,25 @@
         <v>61</v>
       </c>
       <c r="C11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D11" t="s">
         <v>62</v>
       </c>
       <c r="E11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F11" t="s">
         <v>63</v>
       </c>
       <c r="G11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H11" t="s">
         <v>64</v>
       </c>
       <c r="I11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
@@ -1126,25 +1126,25 @@
         <v>65</v>
       </c>
       <c r="C12" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D12" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E12" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F12" t="s">
         <v>66</v>
       </c>
       <c r="G12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H12" t="s">
-        <v>67</v>
+        <v>148</v>
       </c>
       <c r="I12" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
@@ -1152,28 +1152,28 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>67</v>
+      </c>
+      <c r="C13" t="s">
+        <v>93</v>
+      </c>
+      <c r="D13" t="s">
         <v>68</v>
       </c>
-      <c r="C13" t="s">
-        <v>94</v>
-      </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
+        <v>104</v>
+      </c>
+      <c r="F13" t="s">
         <v>69</v>
       </c>
-      <c r="E13" t="s">
-        <v>105</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
+        <v>74</v>
+      </c>
+      <c r="H13" t="s">
         <v>70</v>
       </c>
-      <c r="G13" t="s">
-        <v>75</v>
-      </c>
-      <c r="H13" t="s">
-        <v>71</v>
-      </c>
       <c r="I13" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1192,7 +1192,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B1" t="s">
         <v>13</v>
@@ -1201,13 +1201,13 @@
         <v>14</v>
       </c>
       <c r="D1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E1" t="s">
         <v>114</v>
       </c>
-      <c r="E1" t="s">
-        <v>115</v>
-      </c>
       <c r="F1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -1221,10 +1221,10 @@
         <v>38</v>
       </c>
       <c r="D2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E2" t="s">
         <v>116</v>
-      </c>
-      <c r="E2" t="s">
-        <v>117</v>
       </c>
       <c r="F2" s="2">
         <v>0.58333333333333337</v>
@@ -1235,16 +1235,16 @@
         <v>46184</v>
       </c>
       <c r="B3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F3" s="2">
         <v>0.875</v>
@@ -1258,13 +1258,13 @@
         <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D4" t="s">
+        <v>118</v>
+      </c>
+      <c r="E4" t="s">
         <v>119</v>
-      </c>
-      <c r="E4" t="s">
-        <v>120</v>
       </c>
       <c r="F4" s="2">
         <v>0.58333333333333337</v>
@@ -1281,10 +1281,10 @@
         <v>39</v>
       </c>
       <c r="D5" t="s">
+        <v>120</v>
+      </c>
+      <c r="E5" t="s">
         <v>121</v>
-      </c>
-      <c r="E5" t="s">
-        <v>122</v>
       </c>
       <c r="F5" s="2">
         <v>0.83333333333333337</v>
@@ -1295,16 +1295,16 @@
         <v>46186</v>
       </c>
       <c r="B6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F6" s="2">
         <v>0.83333333333333337</v>
@@ -1315,16 +1315,16 @@
         <v>46186</v>
       </c>
       <c r="B7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F7" s="2">
         <v>0.95833333333333337</v>
@@ -1338,13 +1338,13 @@
         <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F8" s="2">
         <v>0.70833333333333337</v>
@@ -1355,16 +1355,16 @@
         <v>46186</v>
       </c>
       <c r="B9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F9" s="2">
         <v>0.58333333333333337</v>
@@ -1375,16 +1375,16 @@
         <v>46187</v>
       </c>
       <c r="B10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F10" s="2">
         <v>0.75</v>
@@ -1395,16 +1395,16 @@
         <v>46187</v>
       </c>
       <c r="B11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C11" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E11" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F11" s="2">
         <v>0.5</v>
@@ -1415,16 +1415,16 @@
         <v>46187</v>
       </c>
       <c r="B12" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C12" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E12" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F12" s="2">
         <v>0.625</v>
@@ -1435,16 +1435,16 @@
         <v>46187</v>
       </c>
       <c r="B13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C13" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D13" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E13" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F13" s="2">
         <v>0.875</v>
@@ -1455,16 +1455,16 @@
         <v>46188</v>
       </c>
       <c r="B14" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F14" s="2">
         <v>0.70833333333333337</v>
@@ -1475,16 +1475,16 @@
         <v>46188</v>
       </c>
       <c r="B15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C15" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E15" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F15" s="2">
         <v>0.45833333333333331</v>
@@ -1495,16 +1495,16 @@
         <v>46188</v>
       </c>
       <c r="B16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C16" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E16" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F16" s="2">
         <v>0.83333333333333337</v>
@@ -1515,16 +1515,16 @@
         <v>46188</v>
       </c>
       <c r="B17" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C17" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D17" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E17" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F17" s="2">
         <v>0.58333333333333337</v>
@@ -1535,16 +1535,16 @@
         <v>46189</v>
       </c>
       <c r="B18" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C18" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D18" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E18" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F18" s="2">
         <v>0.58333333333333337</v>
@@ -1555,16 +1555,16 @@
         <v>46189</v>
       </c>
       <c r="B19" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C19" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D19" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E19" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F19" s="2">
         <v>0.70833333333333337</v>
@@ -1575,16 +1575,16 @@
         <v>46189</v>
       </c>
       <c r="B20" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C20" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D20" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F20" s="2">
         <v>0.83333333333333337</v>
@@ -1595,16 +1595,16 @@
         <v>46189</v>
       </c>
       <c r="B21" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D21" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E21" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F21" s="2">
         <v>0.95833333333333337</v>
@@ -1615,16 +1615,16 @@
         <v>46190</v>
       </c>
       <c r="B22" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C22" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D22" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E22" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F22" s="2">
         <v>0.75</v>
@@ -1635,16 +1635,16 @@
         <v>46190</v>
       </c>
       <c r="B23" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C23" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D23" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E23" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F23" s="2">
         <v>0.625</v>
@@ -1655,16 +1655,16 @@
         <v>46190</v>
       </c>
       <c r="B24" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C24" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D24" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E24" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F24" s="2">
         <v>0.5</v>
@@ -1675,16 +1675,16 @@
         <v>46190</v>
       </c>
       <c r="B25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C25" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D25" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E25" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F25" s="2">
         <v>0.875</v>
@@ -1695,16 +1695,16 @@
         <v>46191</v>
       </c>
       <c r="B26" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C26" t="s">
         <v>38</v>
       </c>
       <c r="D26" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E26" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F26" s="2">
         <v>0.45833333333333331</v>
@@ -1715,16 +1715,16 @@
         <v>46191</v>
       </c>
       <c r="B27" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C27" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D27" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E27" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F27" s="2">
         <v>0.58333333333333337</v>
@@ -1738,13 +1738,13 @@
         <v>36</v>
       </c>
       <c r="C28" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D28" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E28" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F28" s="2">
         <v>0.70833333333333337</v>
@@ -1758,13 +1758,13 @@
         <v>35</v>
       </c>
       <c r="C29" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D29" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E29" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F29" s="2">
         <v>0.83333333333333337</v>
@@ -1778,13 +1778,13 @@
         <v>37</v>
       </c>
       <c r="C30" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D30" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E30" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F30" s="2">
         <v>0.8125</v>
@@ -1795,16 +1795,16 @@
         <v>46192</v>
       </c>
       <c r="B31" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C31" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D31" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E31" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F31" s="2">
         <v>0.70833333333333337</v>
@@ -1815,16 +1815,16 @@
         <v>46192</v>
       </c>
       <c r="B32" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C32" t="s">
         <v>39</v>
       </c>
       <c r="D32" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E32" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F32" s="2">
         <v>0.91666666666666663</v>
@@ -1838,13 +1838,13 @@
         <v>33</v>
       </c>
       <c r="C33" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D33" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E33" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F33" s="2">
         <v>0.58333333333333337</v>
@@ -1855,16 +1855,16 @@
         <v>46193</v>
       </c>
       <c r="B34" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C34" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D34" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E34" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F34" s="2">
         <v>0.625</v>
@@ -1875,16 +1875,16 @@
         <v>46193</v>
       </c>
       <c r="B35" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C35" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D35" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E35" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F35" s="2">
         <v>0.79166666666666663</v>
@@ -1895,16 +1895,16 @@
         <v>46193</v>
       </c>
       <c r="B36" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C36" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D36" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F36" s="2">
         <v>0.5</v>
@@ -1915,16 +1915,16 @@
         <v>46193</v>
       </c>
       <c r="B37" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C37" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D37" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E37" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F37" s="2">
         <v>0.95833333333333337</v>
@@ -1935,16 +1935,16 @@
         <v>46194</v>
       </c>
       <c r="B38" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C38" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E38" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F38" s="2">
         <v>0.70833333333333337</v>
@@ -1955,16 +1955,16 @@
         <v>46194</v>
       </c>
       <c r="B39" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C39" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D39" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E39" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F39" s="2">
         <v>0.45833333333333331</v>
@@ -1975,16 +1975,16 @@
         <v>46194</v>
       </c>
       <c r="B40" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C40" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D40" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E40" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F40" s="2">
         <v>0.58333333333333337</v>
@@ -1995,16 +1995,16 @@
         <v>46194</v>
       </c>
       <c r="B41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C41" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D41" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E41" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F41" s="2">
         <v>0.83333333333333337</v>
@@ -2015,16 +2015,16 @@
         <v>46195</v>
       </c>
       <c r="B42" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C42" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D42" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E42" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F42" s="2">
         <v>0.79166666666666663</v>
@@ -2035,16 +2035,16 @@
         <v>46195</v>
       </c>
       <c r="B43" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C43" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D43" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E43" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F43" s="2">
         <v>0.66666666666666663</v>
@@ -2055,16 +2055,16 @@
         <v>46195</v>
       </c>
       <c r="B44" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C44" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D44" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E44" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F44" s="2">
         <v>0.5</v>
@@ -2075,16 +2075,16 @@
         <v>46195</v>
       </c>
       <c r="B45" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C45" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D45" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E45" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F45" s="2">
         <v>0.91666666666666663</v>
@@ -2095,16 +2095,16 @@
         <v>46196</v>
       </c>
       <c r="B46" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C46" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D46" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E46" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F46" s="2">
         <v>0.625</v>
@@ -2115,16 +2115,16 @@
         <v>46196</v>
       </c>
       <c r="B47" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C47" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D47" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E47" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F47" s="2">
         <v>0.75</v>
@@ -2135,16 +2135,16 @@
         <v>46196</v>
       </c>
       <c r="B48" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C48" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D48" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E48" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F48" s="2">
         <v>0.5</v>
@@ -2155,16 +2155,16 @@
         <v>46196</v>
       </c>
       <c r="B49" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C49" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D49" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E49" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F49" s="2">
         <v>0.875</v>
@@ -2175,16 +2175,16 @@
         <v>46197</v>
       </c>
       <c r="B50" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C50" t="s">
         <v>37</v>
       </c>
       <c r="D50" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E50" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F50" s="2">
         <v>0.70833333333333337</v>
@@ -2195,16 +2195,16 @@
         <v>46197</v>
       </c>
       <c r="B51" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C51" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D51" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E51" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F51" s="2">
         <v>0.70833333333333337</v>
@@ -2215,16 +2215,16 @@
         <v>46197</v>
       </c>
       <c r="B52" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C52" t="s">
         <v>36</v>
       </c>
       <c r="D52" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E52" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F52" s="2">
         <v>0.58333333333333337</v>
@@ -2235,16 +2235,16 @@
         <v>46197</v>
       </c>
       <c r="B53" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C53" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D53" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E53" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F53" s="2">
         <v>0.58333333333333337</v>
@@ -2255,16 +2255,16 @@
         <v>46197</v>
       </c>
       <c r="B54" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C54" t="s">
         <v>35</v>
       </c>
       <c r="D54" t="s">
+        <v>115</v>
+      </c>
+      <c r="E54" t="s">
         <v>116</v>
-      </c>
-      <c r="E54" t="s">
-        <v>117</v>
       </c>
       <c r="F54" s="2">
         <v>0.83333333333333337</v>
@@ -2278,13 +2278,13 @@
         <v>38</v>
       </c>
       <c r="C55" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D55" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E55" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F55" s="2">
         <v>0.83333333333333337</v>
@@ -2295,16 +2295,16 @@
         <v>46198</v>
       </c>
       <c r="B56" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C56" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D56" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E56" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F56" s="2">
         <v>0.625</v>
@@ -2315,16 +2315,16 @@
         <v>46198</v>
       </c>
       <c r="B57" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C57" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D57" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E57" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F57" s="2">
         <v>0.625</v>
@@ -2335,16 +2335,16 @@
         <v>46198</v>
       </c>
       <c r="B58" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C58" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D58" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E58" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F58" s="2">
         <v>0.75</v>
@@ -2355,16 +2355,16 @@
         <v>46198</v>
       </c>
       <c r="B59" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C59" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D59" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E59" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F59" s="2">
         <v>0.75</v>
@@ -2375,16 +2375,16 @@
         <v>46198</v>
       </c>
       <c r="B60" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C60" t="s">
         <v>33</v>
       </c>
       <c r="D60" t="s">
+        <v>120</v>
+      </c>
+      <c r="E60" t="s">
         <v>121</v>
-      </c>
-      <c r="E60" t="s">
-        <v>122</v>
       </c>
       <c r="F60" s="2">
         <v>0.875</v>
@@ -2398,13 +2398,13 @@
         <v>39</v>
       </c>
       <c r="C61" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D61" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F61" s="2">
         <v>0.875</v>
@@ -2415,16 +2415,16 @@
         <v>46199</v>
       </c>
       <c r="B62" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C62" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D62" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E62" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F62" s="2">
         <v>0.58333333333333337</v>
@@ -2435,16 +2435,16 @@
         <v>46199</v>
       </c>
       <c r="B63" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C63" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D63" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E63" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F63" s="2">
         <v>0.58333333333333337</v>
@@ -2455,16 +2455,16 @@
         <v>46199</v>
       </c>
       <c r="B64" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C64" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D64" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E64" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F64" s="2">
         <v>0.91666666666666663</v>
@@ -2475,16 +2475,16 @@
         <v>46199</v>
       </c>
       <c r="B65" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C65" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D65" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E65" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F65" s="2">
         <v>0.91666666666666663</v>
@@ -2495,16 +2495,16 @@
         <v>46199</v>
       </c>
       <c r="B66" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C66" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D66" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E66" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F66" s="2">
         <v>0.79166666666666663</v>
@@ -2515,16 +2515,16 @@
         <v>46199</v>
       </c>
       <c r="B67" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C67" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D67" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E67" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F67" s="2">
         <v>0.79166666666666663</v>
@@ -2535,16 +2535,16 @@
         <v>46200</v>
       </c>
       <c r="B68" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C68" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D68" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E68" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F68" s="2">
         <v>0.66666666666666663</v>
@@ -2555,16 +2555,16 @@
         <v>46200</v>
       </c>
       <c r="B69" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C69" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D69" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E69" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F69" s="2">
         <v>0.66666666666666663</v>
@@ -2575,16 +2575,16 @@
         <v>46200</v>
       </c>
       <c r="B70" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C70" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D70" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E70" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F70" s="2">
         <v>0.875</v>
@@ -2595,16 +2595,16 @@
         <v>46200</v>
       </c>
       <c r="B71" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C71" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D71" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E71" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F71" s="2">
         <v>0.875</v>
@@ -2615,16 +2615,16 @@
         <v>46200</v>
       </c>
       <c r="B72" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C72" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D72" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E72" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F72" s="2">
         <v>0.77083333333333337</v>
@@ -2635,16 +2635,16 @@
         <v>46200</v>
       </c>
       <c r="B73" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C73" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D73" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E73" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F73" s="2">
         <v>0.77083333333333337</v>

</xml_diff>